<commit_message>
paper run 2026-09-13 23:52
</commit_message>
<xml_diff>
--- a/reports/2026-09-13.xlsx
+++ b/reports/2026-09-13.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,79 +628,111 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>90.81999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По активам</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>90.81999999999999</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>90.81999999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>90.81999999999999</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -722,7 +754,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -744,7 +776,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -766,20 +798,64 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>